<commit_message>
Improve lesson applications and checks for understanding
</commit_message>
<xml_diff>
--- a/resources/Module_Resource_Collection.xlsx
+++ b/resources/Module_Resource_Collection.xlsx
@@ -647,7 +647,7 @@
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="ChecksTable" displayName="ChecksTable" ref="A4:V5" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="ChecksTable" displayName="ChecksTable" ref="A4:V44" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <tableColumns count="22">
     <tableColumn id="1" name="Lesson"/>
     <tableColumn id="2" name="Step"/>
@@ -978,7 +978,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4" ht="26" customHeight="1">
       <c r="A4" s="9" t="inlineStr">
         <is>
@@ -1058,7 +1057,6 @@
         </is>
       </c>
     </row>
-    <row r="11"/>
     <row r="12">
       <c r="A12" s="15" t="inlineStr">
         <is>
@@ -1251,7 +1249,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4" ht="38" customHeight="1">
       <c r="A4" s="35" t="inlineStr">
         <is>
@@ -7892,7 +7889,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4" ht="38" customHeight="1">
       <c r="A4" s="35" t="inlineStr">
         <is>
@@ -10675,7 +10671,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4" ht="38" customHeight="1">
       <c r="A4" s="35" t="inlineStr">
         <is>
@@ -11039,7 +11034,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4" ht="38" customHeight="1">
       <c r="A4" s="35" t="inlineStr">
         <is>
@@ -11525,7 +11519,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4" ht="38" customHeight="1">
       <c r="A4" s="35" t="inlineStr">
         <is>
@@ -17183,7 +17176,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Z22"/>
+  <dimension ref="A1:Z44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -17224,7 +17217,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4" ht="38" customHeight="1">
       <c r="A4" s="35" t="inlineStr">
         <is>
@@ -19120,6 +19112,2074 @@
           <t>Designer approved Lesson 5 preview/content on 2026 to 09 to 13.</t>
         </is>
       </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="n">
+        <v>1</v>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Step .2</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>CFU-1-2-02</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>AG.1; AG.2</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>L1 O2; L1 O3</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>Multiple Choice</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>Why should an Agile team test a small Student Hub update before building every requested feature?</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>It helps the team learn from users and improve the product sooner.</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>It lets the team avoid user feedback until the end.</t>
+        </is>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>It proves the first plan should not change.</t>
+        </is>
+      </c>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>It removes the need for a Product Backlog.</t>
+        </is>
+      </c>
+      <c r="L23" t="inlineStr"/>
+      <c r="M23" t="inlineStr"/>
+      <c r="N23" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="O23" t="inlineStr">
+        <is>
+          <t>Correct. Agile teams use small updates and feedback to learn before making more changes.</t>
+        </is>
+      </c>
+      <c r="P23" t="inlineStr">
+        <is>
+          <t>Not quite. Agile work uses small updates so the team can learn from users and adapt.</t>
+        </is>
+      </c>
+      <c r="Q23" t="inlineStr">
+        <is>
+          <t>R002; R006</t>
+        </is>
+      </c>
+      <c r="R23" t="inlineStr">
+        <is>
+          <t>Understand</t>
+        </is>
+      </c>
+      <c r="S23" t="inlineStr">
+        <is>
+          <t>Added as a second aligned check question for this instructional step.</t>
+        </is>
+      </c>
+      <c r="T23" t="inlineStr"/>
+      <c r="U23" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="V23" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" t="n">
+        <v>1</v>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Step .3</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>CFU-1-3-02</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>AG.1</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>L1 O1</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>Multiple Choice</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>Which action best shows responding to change over following a plan?</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>The team updates the next backlog item after user feedback shows a higher need.</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>The team keeps building the original feature even after users report a barrier.</t>
+        </is>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>The team stops asking users for feedback once the plan is written.</t>
+        </is>
+      </c>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>The team hides new problems so the schedule looks stable.</t>
+        </is>
+      </c>
+      <c r="L24" t="inlineStr"/>
+      <c r="M24" t="inlineStr"/>
+      <c r="N24" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="O24" t="inlineStr">
+        <is>
+          <t>Correct. Agile teams value plans, but they adapt when evidence shows a better path.</t>
+        </is>
+      </c>
+      <c r="P24" t="inlineStr">
+        <is>
+          <t>Review the Agile values. Responding to change means using evidence to adapt the plan.</t>
+        </is>
+      </c>
+      <c r="Q24" t="inlineStr">
+        <is>
+          <t>R006</t>
+        </is>
+      </c>
+      <c r="R24" t="inlineStr">
+        <is>
+          <t>Understand</t>
+        </is>
+      </c>
+      <c r="S24" t="inlineStr">
+        <is>
+          <t>Added as a second aligned check question for this instructional step.</t>
+        </is>
+      </c>
+      <c r="T24" t="inlineStr"/>
+      <c r="U24" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="V24" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" t="n">
+        <v>2</v>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Step .2</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>CFU-2-2-02</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>AG.3; AG.6</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>L2 O1; L2 O2</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>Multiple Choice</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>In Scrum, what does a Sprint help the team do?</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>Create a usable product increment within a short, focused cycle.</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>Delay testing until all lessons are complete.</t>
+        </is>
+      </c>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>Let one person make every product decision alone.</t>
+        </is>
+      </c>
+      <c r="K25" t="inlineStr">
+        <is>
+          <t>Replace teamwork with a fixed checklist.</t>
+        </is>
+      </c>
+      <c r="L25" t="inlineStr"/>
+      <c r="M25" t="inlineStr"/>
+      <c r="N25" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="O25" t="inlineStr">
+        <is>
+          <t>Correct. A Sprint gives the team a short cycle for creating a usable increment.</t>
+        </is>
+      </c>
+      <c r="P25" t="inlineStr">
+        <is>
+          <t>Not quite. A Sprint is a short cycle focused on a useful product increment.</t>
+        </is>
+      </c>
+      <c r="Q25" t="inlineStr">
+        <is>
+          <t>R007</t>
+        </is>
+      </c>
+      <c r="R25" t="inlineStr">
+        <is>
+          <t>Understand</t>
+        </is>
+      </c>
+      <c r="S25" t="inlineStr">
+        <is>
+          <t>Added as a second aligned check question for this instructional step.</t>
+        </is>
+      </c>
+      <c r="T25" t="inlineStr"/>
+      <c r="U25" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="V25" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" t="n">
+        <v>2</v>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Step .3</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>CFU-2-3-01</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>AG.3; AG.6</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>L2 O1; L2 O2</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>Multiple Choice</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>Student testers say the calendar is hard to use on a phone. Which group gives this feedback?</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>Stakeholders</t>
+        </is>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>Scrum Master only</t>
+        </is>
+      </c>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>Developers only</t>
+        </is>
+      </c>
+      <c r="K26" t="inlineStr">
+        <is>
+          <t>Product Backlog</t>
+        </is>
+      </c>
+      <c r="L26" t="inlineStr"/>
+      <c r="M26" t="inlineStr"/>
+      <c r="N26" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="O26" t="inlineStr">
+        <is>
+          <t>Correct. Stakeholders share needs, evidence, and feedback about the product.</t>
+        </is>
+      </c>
+      <c r="P26" t="inlineStr">
+        <is>
+          <t>Review who is inside the Scrum Team and who gives feedback from outside it.</t>
+        </is>
+      </c>
+      <c r="Q26" t="inlineStr">
+        <is>
+          <t>R007</t>
+        </is>
+      </c>
+      <c r="R26" t="inlineStr">
+        <is>
+          <t>Understand</t>
+        </is>
+      </c>
+      <c r="S26" t="inlineStr">
+        <is>
+          <t>Existing approved course check restored to workbook source.</t>
+        </is>
+      </c>
+      <c r="T26" t="inlineStr"/>
+      <c r="U26" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="V26" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" t="n">
+        <v>2</v>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Step .3</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>CFU-2-3-02</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>AG.3; AG.6</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>L2 O1; L2 O2</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>Multiple Choice</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>A Product Owner orders the backlog, and Developers decide how to build the selected work. What does this show?</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>Different Scrum accountabilities support one shared product goal.</t>
+        </is>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>Only the Product Owner is responsible for product quality.</t>
+        </is>
+      </c>
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>Developers should wait for step by step directions.</t>
+        </is>
+      </c>
+      <c r="K27" t="inlineStr">
+        <is>
+          <t>Scrum roles work best when each person works alone.</t>
+        </is>
+      </c>
+      <c r="L27" t="inlineStr"/>
+      <c r="M27" t="inlineStr"/>
+      <c r="N27" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="O27" t="inlineStr">
+        <is>
+          <t>Correct. Scrum accountabilities are different, but they support one shared product goal.</t>
+        </is>
+      </c>
+      <c r="P27" t="inlineStr">
+        <is>
+          <t>Not quite. Scrum uses different accountabilities so the team can work toward one goal.</t>
+        </is>
+      </c>
+      <c r="Q27" t="inlineStr">
+        <is>
+          <t>R007</t>
+        </is>
+      </c>
+      <c r="R27" t="inlineStr">
+        <is>
+          <t>Understand</t>
+        </is>
+      </c>
+      <c r="S27" t="inlineStr">
+        <is>
+          <t>Added as a second aligned check question for this instructional step.</t>
+        </is>
+      </c>
+      <c r="T27" t="inlineStr"/>
+      <c r="U27" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="V27" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" t="n">
+        <v>2</v>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Step .4</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>CFU-2-4-01</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>AG.3; AG.6</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>L2 O3</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>Multiple Choice</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>The Student Hub team needs coding, testing, accessibility, and user feedback skills to finish a calendar improvement. What does this show?</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>The team is cross functional.</t>
+        </is>
+      </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>The Scrum Master assigns all tasks.</t>
+        </is>
+      </c>
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>Stakeholders are Developers.</t>
+        </is>
+      </c>
+      <c r="K28" t="inlineStr">
+        <is>
+          <t>The backlog is finished.</t>
+        </is>
+      </c>
+      <c r="L28" t="inlineStr"/>
+      <c r="M28" t="inlineStr"/>
+      <c r="N28" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="O28" t="inlineStr">
+        <is>
+          <t>Correct. A cross functional team has the skills needed to create a useful Increment.</t>
+        </is>
+      </c>
+      <c r="P28" t="inlineStr">
+        <is>
+          <t>Look for the choice about the team having the skills needed to deliver useful work.</t>
+        </is>
+      </c>
+      <c r="Q28" t="inlineStr">
+        <is>
+          <t>R007; R009</t>
+        </is>
+      </c>
+      <c r="R28" t="inlineStr">
+        <is>
+          <t>Understand</t>
+        </is>
+      </c>
+      <c r="S28" t="inlineStr">
+        <is>
+          <t>Existing approved course check restored to workbook source.</t>
+        </is>
+      </c>
+      <c r="T28" t="inlineStr"/>
+      <c r="U28" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="V28" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" t="n">
+        <v>2</v>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Step .4</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>CFU-2-4-02</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>AG.3; AG.6</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>L2 O3</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>Multiple Choice</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>Why is a cross functional team useful for Student Hub work?</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>The team has the skills needed to deliver value without waiting on many handoffs.</t>
+        </is>
+      </c>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>The team can skip testing because several people are involved.</t>
+        </is>
+      </c>
+      <c r="J29" t="inlineStr">
+        <is>
+          <t>Each person only works inside one narrow role.</t>
+        </is>
+      </c>
+      <c r="K29" t="inlineStr">
+        <is>
+          <t>The team no longer needs a shared goal.</t>
+        </is>
+      </c>
+      <c r="L29" t="inlineStr"/>
+      <c r="M29" t="inlineStr"/>
+      <c r="N29" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="O29" t="inlineStr">
+        <is>
+          <t>Correct. Cross functional teams reduce handoffs because needed skills are on the team.</t>
+        </is>
+      </c>
+      <c r="P29" t="inlineStr">
+        <is>
+          <t>Review the purpose of cross functional teams. The goal is to deliver value with fewer handoffs.</t>
+        </is>
+      </c>
+      <c r="Q29" t="inlineStr">
+        <is>
+          <t>R007; R009</t>
+        </is>
+      </c>
+      <c r="R29" t="inlineStr">
+        <is>
+          <t>Understand</t>
+        </is>
+      </c>
+      <c r="S29" t="inlineStr">
+        <is>
+          <t>Added as a second aligned check question for this instructional step.</t>
+        </is>
+      </c>
+      <c r="T29" t="inlineStr"/>
+      <c r="U29" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="V29" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" t="n">
+        <v>3</v>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Step .2</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>CFU-3-2-02</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>AG.4</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>L3 O1</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>Multiple Choice</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>Which user story keeps the user need and value clear?</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>As a learner, I want assignment dates grouped by course so I can plan my week.</t>
+        </is>
+      </c>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>Add course grouping to the app because it seems useful.</t>
+        </is>
+      </c>
+      <c r="J30" t="inlineStr">
+        <is>
+          <t>Make the page look better before the next Sprint ends.</t>
+        </is>
+      </c>
+      <c r="K30" t="inlineStr">
+        <is>
+          <t>The team should update the assignment screen.</t>
+        </is>
+      </c>
+      <c r="L30" t="inlineStr"/>
+      <c r="M30" t="inlineStr"/>
+      <c r="N30" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="O30" t="inlineStr">
+        <is>
+          <t>Correct. The story names the user, the need, and the value.</t>
+        </is>
+      </c>
+      <c r="P30" t="inlineStr">
+        <is>
+          <t>Look for the user, the need, and the reason the feature matters.</t>
+        </is>
+      </c>
+      <c r="Q30" t="inlineStr">
+        <is>
+          <t>S001; R007</t>
+        </is>
+      </c>
+      <c r="R30" t="inlineStr">
+        <is>
+          <t>Apply</t>
+        </is>
+      </c>
+      <c r="S30" t="inlineStr">
+        <is>
+          <t>Added as a second aligned check question for this instructional step.</t>
+        </is>
+      </c>
+      <c r="T30" t="inlineStr"/>
+      <c r="U30" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="V30" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="A31" t="n">
+        <v>3</v>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Step .3</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>CFU-3-3-01</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>AG.4; AG.10</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>L3 O1; L3 O2</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>Multiple Choice</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>Which acceptance criterion is easiest for another person to test?</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>The calendar should look modern.</t>
+        </is>
+      </c>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>Students will probably like the filter.</t>
+        </is>
+      </c>
+      <c r="J31" t="inlineStr">
+        <is>
+          <t>Keyboard users can reach and use the date filter.</t>
+        </is>
+      </c>
+      <c r="K31" t="inlineStr">
+        <is>
+          <t>The team should build the feature quickly.</t>
+        </is>
+      </c>
+      <c r="L31" t="inlineStr"/>
+      <c r="M31" t="inlineStr"/>
+      <c r="N31" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="O31" t="inlineStr">
+        <is>
+          <t>Correct. A tester can observe whether a keyboard user can reach and use the filter.</t>
+        </is>
+      </c>
+      <c r="P31" t="inlineStr">
+        <is>
+          <t>Choose a product result that can be observed and tested.</t>
+        </is>
+      </c>
+      <c r="Q31" t="inlineStr">
+        <is>
+          <t>R007</t>
+        </is>
+      </c>
+      <c r="R31" t="inlineStr">
+        <is>
+          <t>Understand</t>
+        </is>
+      </c>
+      <c r="S31" t="inlineStr">
+        <is>
+          <t>Existing approved course check restored to workbook source.</t>
+        </is>
+      </c>
+      <c r="T31" t="inlineStr"/>
+      <c r="U31" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="V31" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="A32" t="n">
+        <v>3</v>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Step .3</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>CFU-3-3-02</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>AG.4; AG.10</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>L3 O1; L3 O2</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>Multiple Choice</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>Which acceptance criterion is easiest to test?</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>Given the learner filters by course, then only assignments from that course appear.</t>
+        </is>
+      </c>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>The course filter should feel helpful to most learners.</t>
+        </is>
+      </c>
+      <c r="J32" t="inlineStr">
+        <is>
+          <t>The assignment page should be better than before.</t>
+        </is>
+      </c>
+      <c r="K32" t="inlineStr">
+        <is>
+          <t>Learners should like the updated screen.</t>
+        </is>
+      </c>
+      <c r="L32" t="inlineStr"/>
+      <c r="M32" t="inlineStr"/>
+      <c r="N32" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="O32" t="inlineStr">
+        <is>
+          <t>Correct. A tester can observe whether only the selected course assignments appear.</t>
+        </is>
+      </c>
+      <c r="P32" t="inlineStr">
+        <is>
+          <t>A strong acceptance criterion is specific and testable without guessing.</t>
+        </is>
+      </c>
+      <c r="Q32" t="inlineStr">
+        <is>
+          <t>R007</t>
+        </is>
+      </c>
+      <c r="R32" t="inlineStr">
+        <is>
+          <t>Apply</t>
+        </is>
+      </c>
+      <c r="S32" t="inlineStr">
+        <is>
+          <t>Added as a second aligned check question for this instructional step.</t>
+        </is>
+      </c>
+      <c r="T32" t="inlineStr"/>
+      <c r="U32" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="V32" t="inlineStr"/>
+    </row>
+    <row r="33">
+      <c r="A33" t="n">
+        <v>4</v>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Step .2</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>CFU-4-2-02</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>AG.4; AG.9</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>L4 O1; L4 O2</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>Multiple Choice</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>Which backlog item should move higher when keyboard users cannot open the date filter?</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>Fix the date filter keyboard barrier.</t>
+        </is>
+      </c>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>Change the Student Hub icon color.</t>
+        </is>
+      </c>
+      <c r="J33" t="inlineStr">
+        <is>
+          <t>Add a new welcome message.</t>
+        </is>
+      </c>
+      <c r="K33" t="inlineStr">
+        <is>
+          <t>Write a longer team update.</t>
+        </is>
+      </c>
+      <c r="L33" t="inlineStr"/>
+      <c r="M33" t="inlineStr"/>
+      <c r="N33" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="O33" t="inlineStr">
+        <is>
+          <t>Correct. A barrier that blocks use should move high in the backlog.</t>
+        </is>
+      </c>
+      <c r="P33" t="inlineStr">
+        <is>
+          <t>Think about user value and risk. A feature people cannot use needs attention.</t>
+        </is>
+      </c>
+      <c r="Q33" t="inlineStr">
+        <is>
+          <t>R003; R007</t>
+        </is>
+      </c>
+      <c r="R33" t="inlineStr">
+        <is>
+          <t>Apply</t>
+        </is>
+      </c>
+      <c r="S33" t="inlineStr">
+        <is>
+          <t>Added as a second aligned check question for this instructional step.</t>
+        </is>
+      </c>
+      <c r="T33" t="inlineStr"/>
+      <c r="U33" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="V33" t="inlineStr"/>
+    </row>
+    <row r="34">
+      <c r="A34" t="n">
+        <v>4</v>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Step .3</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>CFU-4-3-02</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>AG.9</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>L4 O1; L4 O2</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>Multiple Choice</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>What should a simple Agile board make visible?</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>What is waiting, in progress, done, and blocked.</t>
+        </is>
+      </c>
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>Only the names of team members.</t>
+        </is>
+      </c>
+      <c r="J34" t="inlineStr">
+        <is>
+          <t>Only the final product grade.</t>
+        </is>
+      </c>
+      <c r="K34" t="inlineStr">
+        <is>
+          <t>Private notes that users cannot see.</t>
+        </is>
+      </c>
+      <c r="L34" t="inlineStr"/>
+      <c r="M34" t="inlineStr"/>
+      <c r="N34" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="O34" t="inlineStr">
+        <is>
+          <t>Correct. A board helps the team see work status and blockers.</t>
+        </is>
+      </c>
+      <c r="P34" t="inlineStr">
+        <is>
+          <t>Review the purpose of visible work. The board should show work status clearly.</t>
+        </is>
+      </c>
+      <c r="Q34" t="inlineStr">
+        <is>
+          <t>R007</t>
+        </is>
+      </c>
+      <c r="R34" t="inlineStr">
+        <is>
+          <t>Understand</t>
+        </is>
+      </c>
+      <c r="S34" t="inlineStr">
+        <is>
+          <t>Added as a second aligned check question for this instructional step.</t>
+        </is>
+      </c>
+      <c r="T34" t="inlineStr"/>
+      <c r="U34" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="V34" t="inlineStr"/>
+    </row>
+    <row r="35">
+      <c r="A35" t="n">
+        <v>5</v>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Step .2</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>CFU-5-2-02</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>AG.5; AG.9</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>L5 O1; L5 O2</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>Multiple Choice</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>What should a Sprint Goal describe?</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>The valuable outcome the team is trying to create in the Sprint.</t>
+        </is>
+      </c>
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>Every small task each person will do.</t>
+        </is>
+      </c>
+      <c r="J35" t="inlineStr">
+        <is>
+          <t>A list of ideas with no priority.</t>
+        </is>
+      </c>
+      <c r="K35" t="inlineStr">
+        <is>
+          <t>A promise that no plan will change.</t>
+        </is>
+      </c>
+      <c r="L35" t="inlineStr"/>
+      <c r="M35" t="inlineStr"/>
+      <c r="N35" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="O35" t="inlineStr">
+        <is>
+          <t>Correct. A Sprint Goal describes the useful outcome, not every task.</t>
+        </is>
+      </c>
+      <c r="P35" t="inlineStr">
+        <is>
+          <t>A Sprint Goal should focus the team on a valuable outcome.</t>
+        </is>
+      </c>
+      <c r="Q35" t="inlineStr">
+        <is>
+          <t>R005; R007</t>
+        </is>
+      </c>
+      <c r="R35" t="inlineStr">
+        <is>
+          <t>Understand</t>
+        </is>
+      </c>
+      <c r="S35" t="inlineStr">
+        <is>
+          <t>Added as a second aligned check question for this instructional step.</t>
+        </is>
+      </c>
+      <c r="T35" t="inlineStr"/>
+      <c r="U35" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="V35" t="inlineStr"/>
+    </row>
+    <row r="36">
+      <c r="A36" t="n">
+        <v>5</v>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Step .3</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>CFU-5-3-02</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>AG.5; AG.10</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>L5 O2</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>Multiple Choice</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>Why should a Sprint Backlog include tasks for testing?</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>Testing is part of the work needed to deliver a quality increment.</t>
+        </is>
+      </c>
+      <c r="I36" t="inlineStr">
+        <is>
+          <t>Testing is only needed after the module ends.</t>
+        </is>
+      </c>
+      <c r="J36" t="inlineStr">
+        <is>
+          <t>Testing replaces the Sprint Goal.</t>
+        </is>
+      </c>
+      <c r="K36" t="inlineStr">
+        <is>
+          <t>Testing should stay hidden from the team plan.</t>
+        </is>
+      </c>
+      <c r="L36" t="inlineStr"/>
+      <c r="M36" t="inlineStr"/>
+      <c r="N36" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="O36" t="inlineStr">
+        <is>
+          <t>Correct. Quality work belongs in the Sprint Backlog so the plan is realistic.</t>
+        </is>
+      </c>
+      <c r="P36" t="inlineStr">
+        <is>
+          <t>Not quite. Testing is part of completing useful, quality work.</t>
+        </is>
+      </c>
+      <c r="Q36" t="inlineStr">
+        <is>
+          <t>R007</t>
+        </is>
+      </c>
+      <c r="R36" t="inlineStr">
+        <is>
+          <t>Understand</t>
+        </is>
+      </c>
+      <c r="S36" t="inlineStr">
+        <is>
+          <t>Added as a second aligned check question for this instructional step.</t>
+        </is>
+      </c>
+      <c r="T36" t="inlineStr"/>
+      <c r="U36" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="V36" t="inlineStr"/>
+    </row>
+    <row r="37">
+      <c r="A37" t="n">
+        <v>5</v>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Step .4</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>CFU-5-4-02</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>AG.5</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>L5 O3</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>Multiple Choice</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>What should the team do if selected work is larger than team capacity?</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>Reduce or split the work so the Sprint plan is realistic.</t>
+        </is>
+      </c>
+      <c r="I37" t="inlineStr">
+        <is>
+          <t>Keep all the work and hope it fits.</t>
+        </is>
+      </c>
+      <c r="J37" t="inlineStr">
+        <is>
+          <t>Remove testing to make more room.</t>
+        </is>
+      </c>
+      <c r="K37" t="inlineStr">
+        <is>
+          <t>Ignore capacity until the Sprint Review.</t>
+        </is>
+      </c>
+      <c r="L37" t="inlineStr"/>
+      <c r="M37" t="inlineStr"/>
+      <c r="N37" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="O37" t="inlineStr">
+        <is>
+          <t>Correct. A realistic Sprint plan fits the team's capacity and protects quality.</t>
+        </is>
+      </c>
+      <c r="P37" t="inlineStr">
+        <is>
+          <t>Review capacity. The team should adjust the plan instead of hiding risk.</t>
+        </is>
+      </c>
+      <c r="Q37" t="inlineStr">
+        <is>
+          <t>R007; R010; S001; S002</t>
+        </is>
+      </c>
+      <c r="R37" t="inlineStr">
+        <is>
+          <t>Apply</t>
+        </is>
+      </c>
+      <c r="S37" t="inlineStr">
+        <is>
+          <t>Added as a second aligned check question for this instructional step.</t>
+        </is>
+      </c>
+      <c r="T37" t="inlineStr"/>
+      <c r="U37" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="V37" t="inlineStr"/>
+    </row>
+    <row r="38">
+      <c r="A38" t="n">
+        <v>6</v>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Step .2</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>CFU-6-2-02</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>AG.3; AG.6; AG.9</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>L6 O1; L6 O2</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>Multiple Choice</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>What is the main purpose of the Daily Scrum?</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>Inspect progress toward the Sprint Goal and adapt the plan.</t>
+        </is>
+      </c>
+      <c r="I38" t="inlineStr">
+        <is>
+          <t>Report every detail to the instructor.</t>
+        </is>
+      </c>
+      <c r="J38" t="inlineStr">
+        <is>
+          <t>Replace the Sprint Review.</t>
+        </is>
+      </c>
+      <c r="K38" t="inlineStr">
+        <is>
+          <t>Choose a new Product Goal each day.</t>
+        </is>
+      </c>
+      <c r="L38" t="inlineStr"/>
+      <c r="M38" t="inlineStr"/>
+      <c r="N38" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="O38" t="inlineStr">
+        <is>
+          <t>Correct. Developers use the Daily Scrum to inspect progress and adapt their plan.</t>
+        </is>
+      </c>
+      <c r="P38" t="inlineStr">
+        <is>
+          <t>Not quite. The Daily Scrum helps Developers inspect progress and adapt.</t>
+        </is>
+      </c>
+      <c r="Q38" t="inlineStr">
+        <is>
+          <t>R007</t>
+        </is>
+      </c>
+      <c r="R38" t="inlineStr">
+        <is>
+          <t>Understand</t>
+        </is>
+      </c>
+      <c r="S38" t="inlineStr">
+        <is>
+          <t>Added as a second aligned check question for this instructional step.</t>
+        </is>
+      </c>
+      <c r="T38" t="inlineStr"/>
+      <c r="U38" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="V38" t="inlineStr"/>
+    </row>
+    <row r="39">
+      <c r="A39" t="n">
+        <v>6</v>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>Step .3</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>CFU-6-3-02</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>AG.3; AG.6; AG.9</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>L6 O1; L6 O2</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>Multiple Choice</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>What should a helpful daily stand up focus on?</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>Progress toward the goal, next work, and anything blocking progress.</t>
+        </is>
+      </c>
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>A long personal update from every team member.</t>
+        </is>
+      </c>
+      <c r="J39" t="inlineStr">
+        <is>
+          <t>Only work that is already done.</t>
+        </is>
+      </c>
+      <c r="K39" t="inlineStr">
+        <is>
+          <t>New features that are not related to the Sprint Goal.</t>
+        </is>
+      </c>
+      <c r="L39" t="inlineStr"/>
+      <c r="M39" t="inlineStr"/>
+      <c r="N39" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="O39" t="inlineStr">
+        <is>
+          <t>Correct. A useful stand up keeps the team focused on progress, next work, and blockers.</t>
+        </is>
+      </c>
+      <c r="P39" t="inlineStr">
+        <is>
+          <t>Review the purpose of a short team check in. It should help the team adapt.</t>
+        </is>
+      </c>
+      <c r="Q39" t="inlineStr">
+        <is>
+          <t>R001; R007</t>
+        </is>
+      </c>
+      <c r="R39" t="inlineStr">
+        <is>
+          <t>Understand</t>
+        </is>
+      </c>
+      <c r="S39" t="inlineStr">
+        <is>
+          <t>Added as a second aligned check question for this instructional step.</t>
+        </is>
+      </c>
+      <c r="T39" t="inlineStr"/>
+      <c r="U39" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="V39" t="inlineStr"/>
+    </row>
+    <row r="40">
+      <c r="A40" t="n">
+        <v>6</v>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Step .4</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>CFU-6-4-02</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>AG.6; AG.9</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>L6 O3</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>Multiple Choice</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>When is a blocker important to raise?</t>
+        </is>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>When it prevents progress toward the Sprint Goal.</t>
+        </is>
+      </c>
+      <c r="I40" t="inlineStr">
+        <is>
+          <t>Only after the Sprint is finished.</t>
+        </is>
+      </c>
+      <c r="J40" t="inlineStr">
+        <is>
+          <t>Only when the blocker is easy to solve alone.</t>
+        </is>
+      </c>
+      <c r="K40" t="inlineStr">
+        <is>
+          <t>When the team wants to avoid changing the plan.</t>
+        </is>
+      </c>
+      <c r="L40" t="inlineStr"/>
+      <c r="M40" t="inlineStr"/>
+      <c r="N40" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="O40" t="inlineStr">
+        <is>
+          <t>Correct. Blockers matter because they can stop progress toward the Sprint Goal.</t>
+        </is>
+      </c>
+      <c r="P40" t="inlineStr">
+        <is>
+          <t>A blocker is important when it slows or stops progress toward the goal.</t>
+        </is>
+      </c>
+      <c r="Q40" t="inlineStr">
+        <is>
+          <t>R023; R007</t>
+        </is>
+      </c>
+      <c r="R40" t="inlineStr">
+        <is>
+          <t>Understand</t>
+        </is>
+      </c>
+      <c r="S40" t="inlineStr">
+        <is>
+          <t>Added as a second aligned check question for this instructional step.</t>
+        </is>
+      </c>
+      <c r="T40" t="inlineStr"/>
+      <c r="U40" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="V40" t="inlineStr"/>
+    </row>
+    <row r="41">
+      <c r="A41" t="n">
+        <v>7</v>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Step .2</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>CFU-7-2-02</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>AG.7</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>L7 O1; L7 O3</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>Multiple Choice</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>What should happen during a Sprint Review?</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>Stakeholders inspect the increment and give product feedback.</t>
+        </is>
+      </c>
+      <c r="I41" t="inlineStr">
+        <is>
+          <t>The team hides unfinished work from users.</t>
+        </is>
+      </c>
+      <c r="J41" t="inlineStr">
+        <is>
+          <t>Developers choose a process improvement without product feedback.</t>
+        </is>
+      </c>
+      <c r="K41" t="inlineStr">
+        <is>
+          <t>The team starts a new Sprint without looking at evidence.</t>
+        </is>
+      </c>
+      <c r="L41" t="inlineStr"/>
+      <c r="M41" t="inlineStr"/>
+      <c r="N41" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="O41" t="inlineStr">
+        <is>
+          <t>Correct. A Sprint Review uses the increment and stakeholder feedback to guide product decisions.</t>
+        </is>
+      </c>
+      <c r="P41" t="inlineStr">
+        <is>
+          <t>Review the Sprint Review purpose. It focuses on the product and feedback.</t>
+        </is>
+      </c>
+      <c r="Q41" t="inlineStr">
+        <is>
+          <t>R014; R007</t>
+        </is>
+      </c>
+      <c r="R41" t="inlineStr">
+        <is>
+          <t>Understand</t>
+        </is>
+      </c>
+      <c r="S41" t="inlineStr">
+        <is>
+          <t>Added as a second aligned check question for this instructional step.</t>
+        </is>
+      </c>
+      <c r="T41" t="inlineStr"/>
+      <c r="U41" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="V41" t="inlineStr"/>
+    </row>
+    <row r="42">
+      <c r="A42" t="n">
+        <v>7</v>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Step .3</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>CFU-7-3-02</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>AG.8</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>L7 O2; L7 O3</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>Multiple Choice</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>What should a team choose during a Sprint Retrospective?</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>One action that can improve how the team works next Sprint.</t>
+        </is>
+      </c>
+      <c r="I42" t="inlineStr">
+        <is>
+          <t>A new product feature with no process discussion.</t>
+        </is>
+      </c>
+      <c r="J42" t="inlineStr">
+        <is>
+          <t>A list of complaints with no next action.</t>
+        </is>
+      </c>
+      <c r="K42" t="inlineStr">
+        <is>
+          <t>A final grade for each team member.</t>
+        </is>
+      </c>
+      <c r="L42" t="inlineStr"/>
+      <c r="M42" t="inlineStr"/>
+      <c r="N42" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="O42" t="inlineStr">
+        <is>
+          <t>Correct. A retrospective should lead to a useful process improvement.</t>
+        </is>
+      </c>
+      <c r="P42" t="inlineStr">
+        <is>
+          <t>Not quite. A retrospective focuses on improving how the team works.</t>
+        </is>
+      </c>
+      <c r="Q42" t="inlineStr">
+        <is>
+          <t>R015; R007</t>
+        </is>
+      </c>
+      <c r="R42" t="inlineStr">
+        <is>
+          <t>Apply</t>
+        </is>
+      </c>
+      <c r="S42" t="inlineStr">
+        <is>
+          <t>Added as a second aligned check question for this instructional step.</t>
+        </is>
+      </c>
+      <c r="T42" t="inlineStr"/>
+      <c r="U42" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="V42" t="inlineStr"/>
+    </row>
+    <row r="43">
+      <c r="A43" t="n">
+        <v>8</v>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>Step .2</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>CFU-8-2-02</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>AG.2; AG.3; AG.7; AG.8; AG.9; AG.10</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>L8 O1</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>Multiple Choice</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>Why should feedback stay connected to the Product Backlog?</t>
+        </is>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>It helps the team use evidence to choose the next improvement.</t>
+        </is>
+      </c>
+      <c r="I43" t="inlineStr">
+        <is>
+          <t>It lets the team ignore the Sprint Goal.</t>
+        </is>
+      </c>
+      <c r="J43" t="inlineStr">
+        <is>
+          <t>It proves every idea should be built right away.</t>
+        </is>
+      </c>
+      <c r="K43" t="inlineStr">
+        <is>
+          <t>It removes the need for review.</t>
+        </is>
+      </c>
+      <c r="L43" t="inlineStr"/>
+      <c r="M43" t="inlineStr"/>
+      <c r="N43" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="O43" t="inlineStr">
+        <is>
+          <t>Correct. Feedback gives evidence the team can use to order future work.</t>
+        </is>
+      </c>
+      <c r="P43" t="inlineStr">
+        <is>
+          <t>Feedback should guide backlog decisions, not sit apart from the work.</t>
+        </is>
+      </c>
+      <c r="Q43" t="inlineStr">
+        <is>
+          <t>R006; R007</t>
+        </is>
+      </c>
+      <c r="R43" t="inlineStr">
+        <is>
+          <t>Understand</t>
+        </is>
+      </c>
+      <c r="S43" t="inlineStr">
+        <is>
+          <t>Added as a second aligned check question for this instructional step.</t>
+        </is>
+      </c>
+      <c r="T43" t="inlineStr"/>
+      <c r="U43" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="V43" t="inlineStr"/>
+    </row>
+    <row r="44">
+      <c r="A44" t="n">
+        <v>8</v>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>Step .3</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>CFU-8-3-02</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>AG.3; AG.10</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>L8 O3</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>Multiple Choice</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>When can the team call a product increment done?</t>
+        </is>
+      </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>When it meets the Definition of Done and the acceptance criteria.</t>
+        </is>
+      </c>
+      <c r="I44" t="inlineStr">
+        <is>
+          <t>When the team runs out of time.</t>
+        </is>
+      </c>
+      <c r="J44" t="inlineStr">
+        <is>
+          <t>When the feature looks complete but has not been tested.</t>
+        </is>
+      </c>
+      <c r="K44" t="inlineStr">
+        <is>
+          <t>When one stakeholder asks for a demo.</t>
+        </is>
+      </c>
+      <c r="L44" t="inlineStr"/>
+      <c r="M44" t="inlineStr"/>
+      <c r="N44" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="O44" t="inlineStr">
+        <is>
+          <t>Correct. Done means the increment meets the shared quality standard and the acceptance criteria.</t>
+        </is>
+      </c>
+      <c r="P44" t="inlineStr">
+        <is>
+          <t>Review the Definition of Done. Work is not done until required quality checks are met.</t>
+        </is>
+      </c>
+      <c r="Q44" t="inlineStr">
+        <is>
+          <t>R007; R012; R016</t>
+        </is>
+      </c>
+      <c r="R44" t="inlineStr">
+        <is>
+          <t>Understand</t>
+        </is>
+      </c>
+      <c r="S44" t="inlineStr">
+        <is>
+          <t>Added as a second aligned check question for this instructional step.</t>
+        </is>
+      </c>
+      <c r="T44" t="inlineStr"/>
+      <c r="U44" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="V44" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -21330,7 +23390,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4" ht="38" customHeight="1">
       <c r="A4" s="35" t="inlineStr">
         <is>

</xml_diff>